<commit_message>
fix(s7b-1a): SIM-001 evidence consistency — validation Pass in E2/E7
deriveValidationStatus SSOT returns Pass (not Not run/Clear) when engine
ran clean on Locked BOQ. E2 adds validation_summary; E7 metadata captures
report snapshot and asserts E2 post_lock consistency. Official SIM-001
re-run from clean hub_it_boq_official DB.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/SPRINT_7B/evidence/SIM-001/E7-export-result/BOQ_Summary_SIM-001_Happy_Path_Project_v1_2026-06-06.xlsx
+++ b/docs/SPRINT_7B/evidence/SIM-001/E7-export-result/BOQ_Summary_SIM-001_Happy_Path_Project_v1_2026-06-06.xlsx
@@ -16,12 +16,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="56">
   <si>
     <t>Generated at</t>
   </si>
   <si>
-    <t>2026-06-06T17:56:14.153Z</t>
+    <t>2026-06-06T18:33:54.874Z</t>
   </si>
   <si>
     <t>Project</t>
@@ -48,7 +48,7 @@
     <t>Handoff Status</t>
   </si>
   <si>
-    <t>Completed · 7/6/2569 00:56:14</t>
+    <t>Completed · 7/6/2569 01:33:54</t>
   </si>
   <si>
     <t>Field</t>
@@ -154,9 +154,6 @@
   </si>
   <si>
     <t>Grand Total (Selling Price)</t>
-  </si>
-  <si>
-    <t>Clear</t>
   </si>
   <si>
     <t>Total Validation Rules</t>
@@ -936,12 +933,12 @@
         <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B2">
         <v>12</v>
@@ -949,7 +946,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -957,7 +954,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -965,15 +962,15 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" t="s">
         <v>50</v>
-      </c>
-      <c r="B5" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -981,7 +978,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -989,18 +986,18 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" t="s">
         <v>54</v>
-      </c>
-      <c r="B8" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>